<commit_message>
update: seed database kategori dan event
</commit_message>
<xml_diff>
--- a/event.xlsx
+++ b/event.xlsx
@@ -1,8 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\PBL smt 4\sisc\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E323977F-E1D3-4EA4-AF88-7E7D9104D8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="event" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -11,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="168">
   <si>
     <t>Polines</t>
   </si>
@@ -202,7 +211,7 @@
     <t>2026-05-05 00:44:52.671362</t>
   </si>
   <si>
-    <t>The 7th Annual International Conference and Exhibition on Indonesian Medical Education and Research </t>
+    <t>The 7th Annual International Conference and Exhibition on Indonesian Medical Education and Research</t>
   </si>
   <si>
     <t>the-7th-annual-international-conference-and-exhibition-on-indonesian-medical-education-and-research-</t>
@@ -416,17 +425,111 @@
   </si>
   <si>
     <t>2026-05-05 00:44:52.727008</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>organizer_id</t>
+  </si>
+  <si>
+    <t>kategori_id</t>
+  </si>
+  <si>
+    <t>kota_id</t>
+  </si>
+  <si>
+    <t>judul</t>
+  </si>
+  <si>
+    <t>slug</t>
+  </si>
+  <si>
+    <t>deskripsi</t>
+  </si>
+  <si>
+    <t>banner_url</t>
+  </si>
+  <si>
+    <t>tanggal_mulai</t>
+  </si>
+  <si>
+    <t>tanggal_selesai</t>
+  </si>
+  <si>
+    <t>detail_lokasi</t>
+  </si>
+  <si>
+    <t>link_eksternal</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>hasil_scraping</t>
+  </si>
+  <si>
+    <t>website_sumber</t>
+  </si>
+  <si>
+    <t>jumlah_tayangan</t>
+  </si>
+  <si>
+    <t>alasan_penolakan</t>
+  </si>
+  <si>
+    <t>dibuat_pada</t>
+  </si>
+  <si>
+    <t>diperbarui_pada</t>
+  </si>
+  <si>
+    <t>syarat_dan_ketentuan</t>
+  </si>
+  <si>
+    <t>batas_registrasi</t>
+  </si>
+  <si>
+    <t>is_event_polines</t>
+  </si>
+  <si>
+    <t>jenis_event</t>
+  </si>
+  <si>
+    <t>tipe_platform</t>
+  </si>
+  <si>
+    <t>tipe_harga</t>
+  </si>
+  <si>
+    <t>harga</t>
+  </si>
+  <si>
+    <t>nama_kontak</t>
+  </si>
+  <si>
+    <t>email_kontak</t>
+  </si>
+  <si>
+    <t>telepon_kontak</t>
+  </si>
+  <si>
+    <t>kuota</t>
+  </si>
+  <si>
+    <t>maks_tiket_per_transaksi</t>
+  </si>
+  <si>
+    <t>satu_akun_satu_transaksi</t>
+  </si>
+  <si>
+    <t>dihapus_pada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="h:mm:ss"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
@@ -444,9 +547,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="1">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="2">
@@ -470,14 +576,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment wrapText="true"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -791,16 +894,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ce6fc980-44b3-410f-982f-1b5ec58c0834}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE6FC980-44B3-410F-982F-1B5EC58C0834}">
   <dimension ref="A1:AG36"/>
-  <sheetFormatPr baseColWidth="12" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="13.140625" defaultRowHeight="18.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="50" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="50" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="28" bestFit="1" customWidth="1"/>
@@ -808,15 +910,13 @@
     <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="50" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="20" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="21" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="22" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="31" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="21" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="26" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="22" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="22" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="19" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="15" bestFit="1" customWidth="1"/>
@@ -825,181 +925,123 @@
     <col min="28" max="28" width="18" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="20" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="31" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="31" bestFit="1" customWidth="1"/>
+    <col min="31" max="32" width="31" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t>organizer_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t>kategori_id</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t>kota_id</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t>judul</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t>slug</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t>deskripsi</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t>banner_url</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t>tanggal_mulai</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr" s="1">
-        <is>
-          <t>tanggal_selesai</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
-        <is>
-          <t>detail_lokasi</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr" s="1">
-        <is>
-          <t>link_eksternal</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr" s="1">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr" s="1">
-        <is>
-          <t>hasil_scraping</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr" s="1">
-        <is>
-          <t>website_sumber</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr" s="1">
-        <is>
-          <t>jumlah_tayangan</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr" s="1">
-        <is>
-          <t>alasan_penolakan</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr" s="1">
-        <is>
-          <t>dibuat_pada</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr" s="1">
-        <is>
-          <t>diperbarui_pada</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr" s="1">
-        <is>
-          <t>syarat_dan_ketentuan</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr" s="1">
-        <is>
-          <t>batas_registrasi</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr" s="1">
-        <is>
-          <t>is_event_polines</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr" s="1">
-        <is>
-          <t>jenis_event</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr" s="1">
-        <is>
-          <t>tipe_platform</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr" s="1">
-        <is>
-          <t>tipe_harga</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr" s="1">
-        <is>
-          <t>harga</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr" s="1">
-        <is>
-          <t>nama_kontak</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr" s="1">
-        <is>
-          <t>email_kontak</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr" s="1">
-        <is>
-          <t>telepon_kontak</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr" s="1">
-        <is>
-          <t>kuota</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr" s="1">
-        <is>
-          <t>maks_tiket_per_transaksi</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr" s="1">
-        <is>
-          <t>satu_akun_satu_transaksi</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr" s="1">
-        <is>
-          <t>dihapus_pada</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" spans="1:33">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
       </c>
       <c r="E2" t="s">
         <v>0</v>
@@ -1029,8 +1071,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:33">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
       <c r="E3" t="s">
@@ -1061,9 +1112,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:33">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
@@ -1093,10 +1153,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:33">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
@@ -1125,10 +1194,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:33">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
       </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
       <c r="E6" t="s">
         <v>0</v>
       </c>
@@ -1157,10 +1235,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:33">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>6</v>
       </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
       <c r="E7" t="s">
         <v>6</v>
       </c>
@@ -1189,10 +1276,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:33">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
@@ -1221,10 +1317,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:33">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
       <c r="E9" t="s">
         <v>12</v>
       </c>
@@ -1253,10 +1358,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:33">
+    <row r="10" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
       <c r="E10" t="s">
         <v>19</v>
       </c>
@@ -1294,10 +1408,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:33">
+    <row r="11" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>10</v>
       </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
       <c r="E11" t="s">
         <v>26</v>
       </c>
@@ -1335,10 +1458,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:33">
+    <row r="12" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>11</v>
       </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
       <c r="E12" t="s">
         <v>30</v>
       </c>
@@ -1376,10 +1508,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:33">
+    <row r="13" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>12</v>
       </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>2</v>
+      </c>
       <c r="E13" t="s">
         <v>34</v>
       </c>
@@ -1417,10 +1558,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:33">
+    <row r="14" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>13</v>
       </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>2</v>
+      </c>
       <c r="E14" t="s">
         <v>38</v>
       </c>
@@ -1458,10 +1608,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:33">
+    <row r="15" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>14</v>
       </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
       <c r="E15" t="s">
         <v>42</v>
       </c>
@@ -1499,10 +1658,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:33">
+    <row r="16" spans="1:33" ht="37" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>15</v>
       </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
       <c r="E16" t="s">
         <v>46</v>
       </c>
@@ -1540,10 +1708,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:33">
+    <row r="17" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>16</v>
       </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
       <c r="E17" t="s">
         <v>51</v>
       </c>
@@ -1581,10 +1755,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:33">
+    <row r="18" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>17</v>
       </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
       <c r="E18" t="s">
         <v>55</v>
       </c>
@@ -1622,10 +1805,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:33">
+    <row r="19" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>18</v>
       </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
       <c r="E19" t="s">
         <v>59</v>
       </c>
@@ -1663,10 +1852,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:33">
+    <row r="20" spans="1:32" ht="55.5" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>19</v>
       </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
       <c r="E20" t="s">
         <v>63</v>
       </c>
@@ -1704,10 +1902,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:33">
+    <row r="21" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>20</v>
       </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
       <c r="E21" t="s">
         <v>67</v>
       </c>
@@ -1745,10 +1952,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:33">
+    <row r="22" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>21</v>
       </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
       <c r="E22" t="s">
         <v>71</v>
       </c>
@@ -1786,10 +1999,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:33">
+    <row r="23" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>22</v>
       </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
       <c r="E23" t="s">
         <v>75</v>
       </c>
@@ -1827,10 +2049,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:33">
+    <row r="24" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>23</v>
       </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
       <c r="E24" t="s">
         <v>80</v>
       </c>
@@ -1868,10 +2099,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:33">
+    <row r="25" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>24</v>
       </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25">
+        <v>2</v>
+      </c>
       <c r="E25" t="s">
         <v>84</v>
       </c>
@@ -1909,10 +2149,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:33">
+    <row r="26" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>25</v>
       </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26">
+        <v>2</v>
+      </c>
       <c r="E26" t="s">
         <v>89</v>
       </c>
@@ -1950,10 +2199,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:33">
+    <row r="27" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>26</v>
       </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>1</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
       <c r="E27" t="s">
         <v>93</v>
       </c>
@@ -1991,10 +2249,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:33">
+    <row r="28" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>27</v>
       </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>2</v>
+      </c>
       <c r="E28" t="s">
         <v>97</v>
       </c>
@@ -2032,10 +2299,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:33">
+    <row r="29" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>28</v>
       </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
       <c r="E29" t="s">
         <v>101</v>
       </c>
@@ -2073,10 +2349,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:33">
+    <row r="30" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>29</v>
       </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
       <c r="E30" t="s">
         <v>106</v>
       </c>
@@ -2114,10 +2399,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:33">
+    <row r="31" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>30</v>
       </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
       <c r="E31" t="s">
         <v>110</v>
       </c>
@@ -2155,10 +2449,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:33">
+    <row r="32" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>31</v>
       </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
       <c r="E32" t="s">
         <v>114</v>
       </c>
@@ -2196,10 +2496,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:33">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>32</v>
       </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
       <c r="E33" t="s">
         <v>118</v>
       </c>
@@ -2237,10 +2546,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:33">
+    <row r="34" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>33</v>
       </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>2</v>
+      </c>
       <c r="E34" t="s">
         <v>122</v>
       </c>
@@ -2278,10 +2596,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:33">
+    <row r="35" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>34</v>
       </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
       <c r="E35" t="s">
         <v>127</v>
       </c>
@@ -2322,10 +2649,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:33">
+    <row r="36" spans="1:32" ht="37" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>35</v>
       </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
       <c r="E36" t="s">
         <v>122</v>
       </c>
@@ -2364,7 +2700,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1" xr:uid="{3036bd9e9-23b9-4345-b53b-ec941b639a77}"/>
+  <autoFilter ref="A1:AG1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>